<commit_message>
Refine honey storefront and connect brand catalog sheet
</commit_message>
<xml_diff>
--- a/templates/honey_store_template.xlsx
+++ b/templates/honey_store_template.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R647b975b18ce4b45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="2" r:id="R9117091ef8174fec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="3" r:id="R73a7f917d0e54cff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ThemeSettings" sheetId="4" r:id="R7dde257d9282473b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductOptions" sheetId="5" r:id="Rcc61c39aef6842ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offers" sheetId="6" r:id="R52bb386fa9ea4e62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="7" r:id="R6bf52cd280ae4af7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rf9ff5239bfb445d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="2" r:id="R25b4440ca2064d39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="3" r:id="Rc05618529e364f1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ThemeSettings" sheetId="4" r:id="R411b1b1c67b4422a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductOptions" sheetId="5" r:id="R33f5a6a1e88546ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offers" sheetId="6" r:id="R63e18dbf3660431c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="7" r:id="R640e042ba2364cbb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -507,7 +507,7 @@
         <x:v>catalog-sweets</x:v>
       </x:c>
       <x:c r="B2" s="13" t="str">
-        <x:v>sweets</x:v>
+        <x:v>thursday</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
         <x:v>الحلويات</x:v>
@@ -518,10 +518,10 @@
       </x:c>
       <x:c r="F2" s="13" t="str"/>
       <x:c r="G2" s="13" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="H2" s="13" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="I2" s="13" t="n">
         <x:v>1</x:v>
@@ -549,10 +549,10 @@
       </x:c>
       <x:c r="F3" s="14" t="str"/>
       <x:c r="G3" s="14" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="H3" s="14" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="I3" s="14" t="n">
         <x:v>2</x:v>
@@ -569,7 +569,7 @@
         <x:v>catalog-brand</x:v>
       </x:c>
       <x:c r="B4" s="13" t="str">
-        <x:v>more</x:v>
+        <x:v>honey</x:v>
       </x:c>
       <x:c r="C4" s="13" t="str">
         <x:v>براند أبو البنات</x:v>
@@ -580,10 +580,10 @@
       </x:c>
       <x:c r="F4" s="13" t="str"/>
       <x:c r="G4" s="13" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="H4" s="13" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="I4" s="13" t="n">
         <x:v>3</x:v>
@@ -600,7 +600,7 @@
         <x:v>catalog-products</x:v>
       </x:c>
       <x:c r="B5" s="16" t="str">
-        <x:v>more</x:v>
+        <x:v>bee</x:v>
       </x:c>
       <x:c r="C5" s="16" t="str">
         <x:v>منتجات</x:v>
@@ -611,7 +611,7 @@
       </x:c>
       <x:c r="F5" s="16" t="str"/>
       <x:c r="G5" s="16" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="H5" s="16" t="str">
         <x:v>FALSE</x:v>
@@ -631,7 +631,7 @@
         <x:v>catalog-abu-albanat</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>more</x:v>
+        <x:v>honey</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
         <x:v>أبو البنات</x:v>
@@ -642,7 +642,7 @@
       </x:c>
       <x:c r="F6" s="16" t="str"/>
       <x:c r="G6" s="16" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="H6" s="16" t="str">
         <x:v>FALSE</x:v>
@@ -676,7 +676,7 @@
         <x:v>TRUE</x:v>
       </x:c>
       <x:c r="H7" s="16" t="str">
-        <x:v>FALSE</x:v>
+        <x:v>TRUE</x:v>
       </x:c>
       <x:c r="I7" s="16" t="n">
         <x:v>6</x:v>
@@ -693,7 +693,7 @@
         <x:v>catalog-beautiful</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
-        <x:v>more</x:v>
+        <x:v>family</x:v>
       </x:c>
       <x:c r="C8" s="16" t="str">
         <x:v>جميل</x:v>
@@ -704,7 +704,7 @@
       </x:c>
       <x:c r="F8" s="16" t="str"/>
       <x:c r="G8" s="16" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="H8" s="16" t="str">
         <x:v>FALSE</x:v>
@@ -724,7 +724,7 @@
         <x:v>catalog-natural</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>more</x:v>
+        <x:v>family</x:v>
       </x:c>
       <x:c r="C9" s="16" t="str">
         <x:v>منتجات طبيعية</x:v>
@@ -735,7 +735,7 @@
       </x:c>
       <x:c r="F9" s="16" t="str"/>
       <x:c r="G9" s="16" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="H9" s="16" t="str">
         <x:v>FALSE</x:v>
@@ -755,7 +755,7 @@
         <x:v>catalog-400</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
-        <x:v>more</x:v>
+        <x:v>family</x:v>
       </x:c>
       <x:c r="C10" s="16" t="str">
         <x:v>٤٠٠</x:v>
@@ -766,7 +766,7 @@
       </x:c>
       <x:c r="F10" s="16" t="str"/>
       <x:c r="G10" s="16" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="H10" s="16" t="str">
         <x:v>FALSE</x:v>
@@ -797,7 +797,7 @@
       </x:c>
       <x:c r="F11" s="16" t="str"/>
       <x:c r="G11" s="16" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="H11" s="16" t="str">
         <x:v>FALSE</x:v>
@@ -817,7 +817,7 @@
         <x:v>couples-blend</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
-        <x:v>mixes</x:v>
+        <x:v>thursday</x:v>
       </x:c>
       <x:c r="C12" s="16" t="str">
         <x:v>خلطة أبو البنات للمتزوجين</x:v>
@@ -2536,7 +2536,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f264fe6a6dc444c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58c0f8da290d4790"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2584,7 +2584,7 @@
         <x:v>العروض</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
-        <x:v>منتجات بسعر خاص</x:v>
+        <x:v>أسعار مميزة</x:v>
       </x:c>
       <x:c r="D2" s="13" t="str"/>
       <x:c r="E2" s="13" t="str">
@@ -2617,10 +2617,10 @@
         <x:v>mixes</x:v>
       </x:c>
       <x:c r="B4" s="13" t="str">
-        <x:v>خلطات المتزوجين</x:v>
+        <x:v>خلطات علاجية</x:v>
       </x:c>
       <x:c r="C4" s="13" t="str">
-        <x:v>استفسار مباشر عن الخلطات</x:v>
+        <x:v>تركيبات من منتجات الخلية</x:v>
       </x:c>
       <x:c r="D4" s="13" t="str"/>
       <x:c r="E4" s="13" t="str">
@@ -2650,13 +2650,13 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="16" t="str">
-        <x:v>sweets</x:v>
+        <x:v>family</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>الحلويات</x:v>
+        <x:v>الأسرة والأطفال</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
-        <x:v>مذاق حلو</x:v>
+        <x:v>اختيارات للعائلة</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str"/>
       <x:c r="E6" s="16" t="str">
@@ -2668,13 +2668,13 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="16" t="str">
-        <x:v>more</x:v>
+        <x:v>thursday</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
-        <x:v>منتجات أخرى</x:v>
+        <x:v>ليلة الخميس</x:v>
       </x:c>
       <x:c r="C7" s="16" t="str">
-        <x:v>اختيارات إضافية</x:v>
+        <x:v>خلطات المتزوجين</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str"/>
       <x:c r="E7" s="16" t="str">
@@ -2692,7 +2692,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64dd5b5adb934481"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c3cd174501a48ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2736,7 +2736,7 @@
         <x:v>restaurant_tagline</x:v>
       </x:c>
       <x:c r="B3" s="14" t="str">
-        <x:v>عسل ومنتجات النحل</x:v>
+        <x:v>اسأل مجرّب ولا تنسى الطبيب</x:v>
       </x:c>
       <x:c r="C3" s="14" t="str">
         <x:v>عبارة قصيرة</x:v>
@@ -2902,7 +2902,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a81fbbf238e4cc8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cd471bfecde4003"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3131,7 +3131,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49f94675f2b9406b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbd4dcb9c8b34c2a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3235,7 +3235,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raceb2e6ab2ca41ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bace6d35de34872"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3324,7 +3324,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b5ab17ba8fa4899"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1966847cff9a4209"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3341,27 +3341,27 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="25" t="str">
-        <x:v>تعليمات كتالوج مناحل أبو البنات</x:v>
+        <x:v>كتالوج براند أبو البنات</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="13" t="str">
-        <x:v>هذا القالب منفصل عن قالب المطعم. استورد نسخة جديدة إلى Google Sheets قبل الإعداد.</x:v>
+        <x:v>الأقسام المعتمدة: العروض، أنواع العسل، خلطات علاجية، منتجات النحل، الأسرة والأطفال، ليلة الخميس.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="14" t="str">
-        <x:v>لا تغيّر أسماء الصفحات أو رؤوس الأعمدة. أضف منتجاتك إلى Products وأقسامك إلى Categories.</x:v>
+        <x:v>استخدم لوحة الإدارة لإضافة المنتجات وصورها. اترك الأقسام دون منتجات ظاهرة لحين توفر أصناف مؤكدة.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="13" t="str">
-        <x:v>السعر: قيمة أكبر من صفر تعني منتجًا مسعّرًا. القيمة 0 تعني «اسأل عن السعر»؛ لا يظهر المنتج كأنه مجاني ولا يمكن إضافته للسلة.</x:v>
+        <x:v>المنتجات ذات السعر صفر للاستفسار عن السعر، وليست مجانية.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="14" t="str">
-        <x:v>سعر المقارنة اختياري، ويجب أن يكون أعلى من السعر الحالي. لا تستخدمه للمنتجات التي تحتاج إلى استفسار.</x:v>
+        <x:v>رابط الصورة يضاف من Drive عبر لوحة الإدارة ولا يوضع في الخلايا يدويًا.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">

</xml_diff>